<commit_message>
Últimos arreglos antes de entrega
</commit_message>
<xml_diff>
--- a/CompletoModelos.xlsx
+++ b/CompletoModelos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mrtor\Desktop\GRU_training\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1820028-1473-450C-A3DA-313D1988E666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B66D78A5-2E3B-4337-B6A8-9FA418570F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15390" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="11055" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Métricas Validación" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="134">
   <si>
     <t>ID Train</t>
   </si>
@@ -484,6 +484,21 @@
   </si>
   <si>
     <t>103,994 W</t>
+  </si>
+  <si>
+    <t>Tipo de evaluación</t>
+  </si>
+  <si>
+    <t>HIL (INT8, dataset SISIFO, completo)</t>
+  </si>
+  <si>
+    <t>Producción real (completo)</t>
+  </si>
+  <si>
+    <t>Producción real (diurno, G &gt; 70 W/m^2)</t>
+  </si>
+  <si>
+    <t>HIL (Datos reales de mayo)</t>
   </si>
 </sst>
 </file>
@@ -1479,7 +1494,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="217">
+  <cellXfs count="224">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -1727,195 +1742,210 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="5" fillId="14" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="59" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="48" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="17" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2396,32 +2426,32 @@
   <sheetData>
     <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="D3" s="181" t="s">
+      <c r="D3" s="191" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="182"/>
-      <c r="F3" s="182"/>
-      <c r="G3" s="182"/>
-      <c r="H3" s="183"/>
-      <c r="I3" s="184" t="s">
+      <c r="E3" s="192"/>
+      <c r="F3" s="192"/>
+      <c r="G3" s="192"/>
+      <c r="H3" s="193"/>
+      <c r="I3" s="194" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="185"/>
-      <c r="K3" s="185"/>
-      <c r="L3" s="185"/>
-      <c r="M3" s="185"/>
-      <c r="N3" s="185"/>
-      <c r="O3" s="185"/>
-      <c r="P3" s="185"/>
-      <c r="Q3" s="186"/>
-      <c r="R3" s="191" t="s">
+      <c r="J3" s="195"/>
+      <c r="K3" s="195"/>
+      <c r="L3" s="195"/>
+      <c r="M3" s="195"/>
+      <c r="N3" s="195"/>
+      <c r="O3" s="195"/>
+      <c r="P3" s="195"/>
+      <c r="Q3" s="196"/>
+      <c r="R3" s="198" t="s">
         <v>20</v>
       </c>
-      <c r="S3" s="192"/>
-      <c r="T3" s="192"/>
-      <c r="U3" s="192"/>
-      <c r="V3" s="192"/>
-      <c r="W3" s="193"/>
+      <c r="S3" s="199"/>
+      <c r="T3" s="199"/>
+      <c r="U3" s="199"/>
+      <c r="V3" s="199"/>
+      <c r="W3" s="187"/>
     </row>
     <row r="4" spans="1:23" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B4" s="19" t="s">
@@ -2472,16 +2502,16 @@
       <c r="Q4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="R4" s="194"/>
-      <c r="S4" s="195"/>
-      <c r="T4" s="195"/>
-      <c r="U4" s="195"/>
-      <c r="V4" s="195"/>
-      <c r="W4" s="196"/>
+      <c r="R4" s="200"/>
+      <c r="S4" s="201"/>
+      <c r="T4" s="201"/>
+      <c r="U4" s="201"/>
+      <c r="V4" s="201"/>
+      <c r="W4" s="189"/>
     </row>
     <row r="5" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
-      <c r="B5" s="187" t="s">
+      <c r="B5" s="197" t="s">
         <v>15</v>
       </c>
       <c r="C5" s="5" t="s">
@@ -2529,18 +2559,18 @@
       <c r="Q5" s="16">
         <v>1E-3</v>
       </c>
-      <c r="R5" s="179" t="s">
+      <c r="R5" s="186" t="s">
         <v>38</v>
       </c>
-      <c r="S5" s="174"/>
-      <c r="T5" s="174"/>
-      <c r="U5" s="174"/>
-      <c r="V5" s="174"/>
-      <c r="W5" s="175"/>
+      <c r="S5" s="178"/>
+      <c r="T5" s="178"/>
+      <c r="U5" s="178"/>
+      <c r="V5" s="178"/>
+      <c r="W5" s="179"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
-      <c r="B6" s="188"/>
+      <c r="B6" s="164"/>
       <c r="C6" s="5" t="s">
         <v>12</v>
       </c>
@@ -2586,16 +2616,16 @@
       <c r="Q6" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R6" s="167"/>
-      <c r="S6" s="168"/>
-      <c r="T6" s="168"/>
-      <c r="U6" s="168"/>
-      <c r="V6" s="168"/>
-      <c r="W6" s="169"/>
+      <c r="R6" s="180"/>
+      <c r="S6" s="181"/>
+      <c r="T6" s="181"/>
+      <c r="U6" s="181"/>
+      <c r="V6" s="181"/>
+      <c r="W6" s="182"/>
     </row>
     <row r="7" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7"/>
-      <c r="B7" s="189"/>
+      <c r="B7" s="190"/>
       <c r="C7" s="13" t="s">
         <v>14</v>
       </c>
@@ -2641,16 +2671,16 @@
       <c r="Q7" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R7" s="170"/>
-      <c r="S7" s="171"/>
-      <c r="T7" s="171"/>
-      <c r="U7" s="171"/>
-      <c r="V7" s="171"/>
-      <c r="W7" s="172"/>
+      <c r="R7" s="183"/>
+      <c r="S7" s="184"/>
+      <c r="T7" s="184"/>
+      <c r="U7" s="184"/>
+      <c r="V7" s="184"/>
+      <c r="W7" s="185"/>
     </row>
     <row r="8" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
-      <c r="B8" s="190" t="s">
+      <c r="B8" s="163" t="s">
         <v>24</v>
       </c>
       <c r="C8" s="5" t="s">
@@ -2698,18 +2728,18 @@
       <c r="Q8" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R8" s="179" t="s">
+      <c r="R8" s="186" t="s">
         <v>38</v>
       </c>
-      <c r="S8" s="174"/>
-      <c r="T8" s="174"/>
-      <c r="U8" s="174"/>
-      <c r="V8" s="174"/>
-      <c r="W8" s="175"/>
+      <c r="S8" s="178"/>
+      <c r="T8" s="178"/>
+      <c r="U8" s="178"/>
+      <c r="V8" s="178"/>
+      <c r="W8" s="179"/>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
-      <c r="B9" s="188"/>
+      <c r="B9" s="164"/>
       <c r="C9" s="5" t="s">
         <v>12</v>
       </c>
@@ -2755,16 +2785,16 @@
       <c r="Q9" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R9" s="167"/>
-      <c r="S9" s="168"/>
-      <c r="T9" s="168"/>
-      <c r="U9" s="168"/>
-      <c r="V9" s="168"/>
-      <c r="W9" s="169"/>
+      <c r="R9" s="180"/>
+      <c r="S9" s="181"/>
+      <c r="T9" s="181"/>
+      <c r="U9" s="181"/>
+      <c r="V9" s="181"/>
+      <c r="W9" s="182"/>
     </row>
     <row r="10" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7"/>
-      <c r="B10" s="189"/>
+      <c r="B10" s="190"/>
       <c r="C10" s="5" t="s">
         <v>14</v>
       </c>
@@ -2810,15 +2840,15 @@
       <c r="Q10" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R10" s="170"/>
-      <c r="S10" s="171"/>
-      <c r="T10" s="171"/>
-      <c r="U10" s="171"/>
-      <c r="V10" s="171"/>
-      <c r="W10" s="172"/>
+      <c r="R10" s="183"/>
+      <c r="S10" s="184"/>
+      <c r="T10" s="184"/>
+      <c r="U10" s="184"/>
+      <c r="V10" s="184"/>
+      <c r="W10" s="185"/>
     </row>
     <row r="11" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="190" t="s">
+      <c r="B11" s="163" t="s">
         <v>34</v>
       </c>
       <c r="C11" s="28" t="s">
@@ -2866,17 +2896,17 @@
       <c r="Q11" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R11" s="179" t="s">
+      <c r="R11" s="186" t="s">
         <v>38</v>
       </c>
-      <c r="S11" s="174"/>
-      <c r="T11" s="174"/>
-      <c r="U11" s="174"/>
-      <c r="V11" s="174"/>
-      <c r="W11" s="175"/>
+      <c r="S11" s="178"/>
+      <c r="T11" s="178"/>
+      <c r="U11" s="178"/>
+      <c r="V11" s="178"/>
+      <c r="W11" s="179"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B12" s="188"/>
+      <c r="B12" s="164"/>
       <c r="C12" s="25" t="s">
         <v>12</v>
       </c>
@@ -2922,15 +2952,15 @@
       <c r="Q12" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R12" s="167"/>
-      <c r="S12" s="168"/>
-      <c r="T12" s="168"/>
-      <c r="U12" s="168"/>
-      <c r="V12" s="168"/>
-      <c r="W12" s="169"/>
+      <c r="R12" s="180"/>
+      <c r="S12" s="181"/>
+      <c r="T12" s="181"/>
+      <c r="U12" s="181"/>
+      <c r="V12" s="181"/>
+      <c r="W12" s="182"/>
     </row>
     <row r="13" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="188"/>
+      <c r="B13" s="164"/>
       <c r="C13" s="26" t="s">
         <v>14</v>
       </c>
@@ -2976,15 +3006,15 @@
       <c r="Q13" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R13" s="170"/>
-      <c r="S13" s="171"/>
-      <c r="T13" s="171"/>
-      <c r="U13" s="171"/>
-      <c r="V13" s="171"/>
-      <c r="W13" s="172"/>
+      <c r="R13" s="183"/>
+      <c r="S13" s="184"/>
+      <c r="T13" s="184"/>
+      <c r="U13" s="184"/>
+      <c r="V13" s="184"/>
+      <c r="W13" s="185"/>
     </row>
     <row r="14" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="190" t="s">
+      <c r="B14" s="163" t="s">
         <v>36</v>
       </c>
       <c r="C14" s="19" t="s">
@@ -3032,17 +3062,17 @@
       <c r="Q14" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R14" s="179" t="s">
+      <c r="R14" s="186" t="s">
         <v>37</v>
       </c>
-      <c r="S14" s="174"/>
-      <c r="T14" s="174"/>
-      <c r="U14" s="174"/>
-      <c r="V14" s="174"/>
-      <c r="W14" s="175"/>
+      <c r="S14" s="178"/>
+      <c r="T14" s="178"/>
+      <c r="U14" s="178"/>
+      <c r="V14" s="178"/>
+      <c r="W14" s="179"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B15" s="188"/>
+      <c r="B15" s="164"/>
       <c r="C15" s="29" t="s">
         <v>12</v>
       </c>
@@ -3088,15 +3118,15 @@
       <c r="Q15" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R15" s="167"/>
-      <c r="S15" s="168"/>
-      <c r="T15" s="168"/>
-      <c r="U15" s="168"/>
-      <c r="V15" s="168"/>
-      <c r="W15" s="169"/>
+      <c r="R15" s="180"/>
+      <c r="S15" s="181"/>
+      <c r="T15" s="181"/>
+      <c r="U15" s="181"/>
+      <c r="V15" s="181"/>
+      <c r="W15" s="182"/>
     </row>
     <row r="16" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="189"/>
+      <c r="B16" s="190"/>
       <c r="C16" s="30" t="s">
         <v>14</v>
       </c>
@@ -3142,16 +3172,16 @@
       <c r="Q16" s="3">
         <v>1E-3</v>
       </c>
-      <c r="R16" s="170"/>
-      <c r="S16" s="171"/>
-      <c r="T16" s="171"/>
-      <c r="U16" s="171"/>
-      <c r="V16" s="171"/>
-      <c r="W16" s="172"/>
+      <c r="R16" s="183"/>
+      <c r="S16" s="184"/>
+      <c r="T16" s="184"/>
+      <c r="U16" s="184"/>
+      <c r="V16" s="184"/>
+      <c r="W16" s="185"/>
     </row>
     <row r="17" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
-      <c r="B17" s="193" t="s">
+      <c r="B17" s="187" t="s">
         <v>44</v>
       </c>
       <c r="C17" s="29" t="s">
@@ -3199,18 +3229,18 @@
       <c r="Q17" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R17" s="174" t="s">
+      <c r="R17" s="178" t="s">
         <v>43</v>
       </c>
-      <c r="S17" s="174"/>
-      <c r="T17" s="174"/>
-      <c r="U17" s="174"/>
-      <c r="V17" s="174"/>
-      <c r="W17" s="175"/>
+      <c r="S17" s="178"/>
+      <c r="T17" s="178"/>
+      <c r="U17" s="178"/>
+      <c r="V17" s="178"/>
+      <c r="W17" s="179"/>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
-      <c r="B18" s="197"/>
+      <c r="B18" s="188"/>
       <c r="C18" s="29" t="s">
         <v>12</v>
       </c>
@@ -3256,16 +3286,16 @@
       <c r="Q18" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R18" s="168"/>
-      <c r="S18" s="168"/>
-      <c r="T18" s="168"/>
-      <c r="U18" s="168"/>
-      <c r="V18" s="168"/>
-      <c r="W18" s="169"/>
+      <c r="R18" s="181"/>
+      <c r="S18" s="181"/>
+      <c r="T18" s="181"/>
+      <c r="U18" s="181"/>
+      <c r="V18" s="181"/>
+      <c r="W18" s="182"/>
     </row>
     <row r="19" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="7"/>
-      <c r="B19" s="196"/>
+      <c r="B19" s="189"/>
       <c r="C19" s="30" t="s">
         <v>14</v>
       </c>
@@ -3311,16 +3341,16 @@
       <c r="Q19" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R19" s="171"/>
-      <c r="S19" s="171"/>
-      <c r="T19" s="171"/>
-      <c r="U19" s="171"/>
-      <c r="V19" s="171"/>
-      <c r="W19" s="172"/>
+      <c r="R19" s="184"/>
+      <c r="S19" s="184"/>
+      <c r="T19" s="184"/>
+      <c r="U19" s="184"/>
+      <c r="V19" s="184"/>
+      <c r="W19" s="185"/>
     </row>
     <row r="20" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
-      <c r="B20" s="190" t="s">
+      <c r="B20" s="163" t="s">
         <v>46</v>
       </c>
       <c r="C20" s="29" t="s">
@@ -3368,18 +3398,18 @@
       <c r="Q20" s="35">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R20" s="173" t="s">
+      <c r="R20" s="177" t="s">
         <v>45</v>
       </c>
-      <c r="S20" s="174"/>
-      <c r="T20" s="174"/>
-      <c r="U20" s="174"/>
-      <c r="V20" s="174"/>
-      <c r="W20" s="175"/>
+      <c r="S20" s="178"/>
+      <c r="T20" s="178"/>
+      <c r="U20" s="178"/>
+      <c r="V20" s="178"/>
+      <c r="W20" s="179"/>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
-      <c r="B21" s="188"/>
+      <c r="B21" s="164"/>
       <c r="C21" s="29" t="s">
         <v>12</v>
       </c>
@@ -3425,16 +3455,16 @@
       <c r="Q21" s="36">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R21" s="167"/>
-      <c r="S21" s="168"/>
-      <c r="T21" s="168"/>
-      <c r="U21" s="168"/>
-      <c r="V21" s="168"/>
-      <c r="W21" s="169"/>
+      <c r="R21" s="180"/>
+      <c r="S21" s="181"/>
+      <c r="T21" s="181"/>
+      <c r="U21" s="181"/>
+      <c r="V21" s="181"/>
+      <c r="W21" s="182"/>
     </row>
     <row r="22" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="7"/>
-      <c r="B22" s="189"/>
+      <c r="B22" s="190"/>
       <c r="C22" s="30" t="s">
         <v>14</v>
       </c>
@@ -3480,16 +3510,16 @@
       <c r="Q22" s="37">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R22" s="170"/>
-      <c r="S22" s="171"/>
-      <c r="T22" s="171"/>
-      <c r="U22" s="171"/>
-      <c r="V22" s="171"/>
-      <c r="W22" s="172"/>
+      <c r="R22" s="183"/>
+      <c r="S22" s="184"/>
+      <c r="T22" s="184"/>
+      <c r="U22" s="184"/>
+      <c r="V22" s="184"/>
+      <c r="W22" s="185"/>
     </row>
     <row r="23" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A23" s="58"/>
-      <c r="B23" s="162" t="s">
+      <c r="B23" s="165" t="s">
         <v>15</v>
       </c>
       <c r="C23" s="19" t="s">
@@ -3537,18 +3567,18 @@
       <c r="Q23" s="9">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R23" s="173" t="s">
+      <c r="R23" s="177" t="s">
         <v>53</v>
       </c>
-      <c r="S23" s="174"/>
-      <c r="T23" s="174"/>
-      <c r="U23" s="174"/>
-      <c r="V23" s="174"/>
-      <c r="W23" s="175"/>
+      <c r="S23" s="178"/>
+      <c r="T23" s="178"/>
+      <c r="U23" s="178"/>
+      <c r="V23" s="178"/>
+      <c r="W23" s="179"/>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="58"/>
-      <c r="B24" s="163"/>
+      <c r="B24" s="166"/>
       <c r="C24" s="29" t="s">
         <v>12</v>
       </c>
@@ -3594,16 +3624,16 @@
       <c r="Q24" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R24" s="167"/>
-      <c r="S24" s="168"/>
-      <c r="T24" s="168"/>
-      <c r="U24" s="168"/>
-      <c r="V24" s="168"/>
-      <c r="W24" s="169"/>
+      <c r="R24" s="180"/>
+      <c r="S24" s="181"/>
+      <c r="T24" s="181"/>
+      <c r="U24" s="181"/>
+      <c r="V24" s="181"/>
+      <c r="W24" s="182"/>
     </row>
     <row r="25" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="58"/>
-      <c r="B25" s="166"/>
+      <c r="B25" s="167"/>
       <c r="C25" s="30" t="s">
         <v>14</v>
       </c>
@@ -3649,16 +3679,16 @@
       <c r="Q25" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R25" s="170"/>
-      <c r="S25" s="171"/>
-      <c r="T25" s="171"/>
-      <c r="U25" s="171"/>
-      <c r="V25" s="171"/>
-      <c r="W25" s="172"/>
+      <c r="R25" s="183"/>
+      <c r="S25" s="184"/>
+      <c r="T25" s="184"/>
+      <c r="U25" s="184"/>
+      <c r="V25" s="184"/>
+      <c r="W25" s="185"/>
     </row>
     <row r="26" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A26" s="58"/>
-      <c r="B26" s="162" t="s">
+      <c r="B26" s="165" t="s">
         <v>24</v>
       </c>
       <c r="C26" s="19" t="s">
@@ -3706,18 +3736,18 @@
       <c r="Q26" s="35">
         <v>1E-3</v>
       </c>
-      <c r="R26" s="179" t="s">
+      <c r="R26" s="186" t="s">
         <v>57</v>
       </c>
-      <c r="S26" s="174"/>
-      <c r="T26" s="174"/>
-      <c r="U26" s="174"/>
-      <c r="V26" s="174"/>
-      <c r="W26" s="175"/>
+      <c r="S26" s="178"/>
+      <c r="T26" s="178"/>
+      <c r="U26" s="178"/>
+      <c r="V26" s="178"/>
+      <c r="W26" s="179"/>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="58"/>
-      <c r="B27" s="163"/>
+      <c r="B27" s="166"/>
       <c r="C27" s="29" t="s">
         <v>12</v>
       </c>
@@ -3763,16 +3793,16 @@
       <c r="Q27" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R27" s="167"/>
-      <c r="S27" s="168"/>
-      <c r="T27" s="168"/>
-      <c r="U27" s="168"/>
-      <c r="V27" s="168"/>
-      <c r="W27" s="169"/>
+      <c r="R27" s="180"/>
+      <c r="S27" s="181"/>
+      <c r="T27" s="181"/>
+      <c r="U27" s="181"/>
+      <c r="V27" s="181"/>
+      <c r="W27" s="182"/>
     </row>
     <row r="28" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="58"/>
-      <c r="B28" s="166"/>
+      <c r="B28" s="167"/>
       <c r="C28" s="30" t="s">
         <v>14</v>
       </c>
@@ -3818,16 +3848,16 @@
       <c r="Q28" s="37">
         <v>1E-3</v>
       </c>
-      <c r="R28" s="170"/>
-      <c r="S28" s="171"/>
-      <c r="T28" s="171"/>
-      <c r="U28" s="171"/>
-      <c r="V28" s="171"/>
-      <c r="W28" s="172"/>
+      <c r="R28" s="183"/>
+      <c r="S28" s="184"/>
+      <c r="T28" s="184"/>
+      <c r="U28" s="184"/>
+      <c r="V28" s="184"/>
+      <c r="W28" s="185"/>
     </row>
     <row r="29" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A29" s="59"/>
-      <c r="B29" s="162" t="s">
+      <c r="B29" s="165" t="s">
         <v>34</v>
       </c>
       <c r="C29" s="28" t="s">
@@ -3875,18 +3905,18 @@
       <c r="Q29" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R29" s="173" t="s">
+      <c r="R29" s="177" t="s">
         <v>60</v>
       </c>
-      <c r="S29" s="174"/>
-      <c r="T29" s="174"/>
-      <c r="U29" s="174"/>
-      <c r="V29" s="174"/>
-      <c r="W29" s="175"/>
+      <c r="S29" s="178"/>
+      <c r="T29" s="178"/>
+      <c r="U29" s="178"/>
+      <c r="V29" s="178"/>
+      <c r="W29" s="179"/>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="58"/>
-      <c r="B30" s="163"/>
+      <c r="B30" s="166"/>
       <c r="C30" s="25" t="s">
         <v>12</v>
       </c>
@@ -3932,16 +3962,16 @@
       <c r="Q30" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R30" s="167"/>
-      <c r="S30" s="168"/>
-      <c r="T30" s="168"/>
-      <c r="U30" s="168"/>
-      <c r="V30" s="168"/>
-      <c r="W30" s="169"/>
+      <c r="R30" s="180"/>
+      <c r="S30" s="181"/>
+      <c r="T30" s="181"/>
+      <c r="U30" s="181"/>
+      <c r="V30" s="181"/>
+      <c r="W30" s="182"/>
     </row>
     <row r="31" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="58"/>
-      <c r="B31" s="166"/>
+      <c r="B31" s="167"/>
       <c r="C31" s="42" t="s">
         <v>14</v>
       </c>
@@ -3987,16 +4017,16 @@
       <c r="Q31" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R31" s="170"/>
-      <c r="S31" s="171"/>
-      <c r="T31" s="171"/>
-      <c r="U31" s="171"/>
-      <c r="V31" s="171"/>
-      <c r="W31" s="172"/>
+      <c r="R31" s="183"/>
+      <c r="S31" s="184"/>
+      <c r="T31" s="184"/>
+      <c r="U31" s="184"/>
+      <c r="V31" s="184"/>
+      <c r="W31" s="185"/>
     </row>
     <row r="32" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A32" s="59"/>
-      <c r="B32" s="162" t="s">
+      <c r="B32" s="165" t="s">
         <v>36</v>
       </c>
       <c r="C32" s="28" t="s">
@@ -4044,18 +4074,18 @@
       <c r="Q32" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R32" s="179" t="s">
+      <c r="R32" s="186" t="s">
         <v>61</v>
       </c>
-      <c r="S32" s="174"/>
-      <c r="T32" s="174"/>
-      <c r="U32" s="174"/>
-      <c r="V32" s="174"/>
-      <c r="W32" s="175"/>
+      <c r="S32" s="178"/>
+      <c r="T32" s="178"/>
+      <c r="U32" s="178"/>
+      <c r="V32" s="178"/>
+      <c r="W32" s="179"/>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" s="59"/>
-      <c r="B33" s="163"/>
+      <c r="B33" s="166"/>
       <c r="C33" s="25" t="s">
         <v>12</v>
       </c>
@@ -4101,16 +4131,16 @@
       <c r="Q33" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R33" s="167"/>
-      <c r="S33" s="168"/>
-      <c r="T33" s="168"/>
-      <c r="U33" s="168"/>
-      <c r="V33" s="168"/>
-      <c r="W33" s="169"/>
+      <c r="R33" s="180"/>
+      <c r="S33" s="181"/>
+      <c r="T33" s="181"/>
+      <c r="U33" s="181"/>
+      <c r="V33" s="181"/>
+      <c r="W33" s="182"/>
     </row>
     <row r="34" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="59"/>
-      <c r="B34" s="166"/>
+      <c r="B34" s="167"/>
       <c r="C34" s="42" t="s">
         <v>14</v>
       </c>
@@ -4156,16 +4186,16 @@
       <c r="Q34" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R34" s="170"/>
-      <c r="S34" s="171"/>
-      <c r="T34" s="171"/>
-      <c r="U34" s="171"/>
-      <c r="V34" s="171"/>
-      <c r="W34" s="172"/>
+      <c r="R34" s="183"/>
+      <c r="S34" s="184"/>
+      <c r="T34" s="184"/>
+      <c r="U34" s="184"/>
+      <c r="V34" s="184"/>
+      <c r="W34" s="185"/>
     </row>
     <row r="35" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A35" s="58"/>
-      <c r="B35" s="162" t="s">
+      <c r="B35" s="165" t="s">
         <v>44</v>
       </c>
       <c r="C35" s="25" t="s">
@@ -4213,18 +4243,18 @@
       <c r="Q35" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R35" s="173" t="s">
+      <c r="R35" s="177" t="s">
         <v>63</v>
       </c>
-      <c r="S35" s="174"/>
-      <c r="T35" s="174"/>
-      <c r="U35" s="174"/>
-      <c r="V35" s="174"/>
-      <c r="W35" s="175"/>
+      <c r="S35" s="178"/>
+      <c r="T35" s="178"/>
+      <c r="U35" s="178"/>
+      <c r="V35" s="178"/>
+      <c r="W35" s="179"/>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A36" s="58"/>
-      <c r="B36" s="163"/>
+      <c r="B36" s="166"/>
       <c r="C36" s="25" t="s">
         <v>12</v>
       </c>
@@ -4270,16 +4300,16 @@
       <c r="Q36" s="36">
         <v>1E-3</v>
       </c>
-      <c r="R36" s="167"/>
-      <c r="S36" s="168"/>
-      <c r="T36" s="168"/>
-      <c r="U36" s="168"/>
-      <c r="V36" s="168"/>
-      <c r="W36" s="169"/>
+      <c r="R36" s="180"/>
+      <c r="S36" s="181"/>
+      <c r="T36" s="181"/>
+      <c r="U36" s="181"/>
+      <c r="V36" s="181"/>
+      <c r="W36" s="182"/>
     </row>
     <row r="37" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="58"/>
-      <c r="B37" s="166"/>
+      <c r="B37" s="167"/>
       <c r="C37" s="30" t="s">
         <v>14</v>
       </c>
@@ -4325,16 +4355,16 @@
       <c r="Q37" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R37" s="170"/>
-      <c r="S37" s="171"/>
-      <c r="T37" s="171"/>
-      <c r="U37" s="171"/>
-      <c r="V37" s="171"/>
-      <c r="W37" s="172"/>
+      <c r="R37" s="183"/>
+      <c r="S37" s="184"/>
+      <c r="T37" s="184"/>
+      <c r="U37" s="184"/>
+      <c r="V37" s="184"/>
+      <c r="W37" s="185"/>
     </row>
     <row r="38" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A38" s="59"/>
-      <c r="B38" s="162" t="s">
+      <c r="B38" s="165" t="s">
         <v>46</v>
       </c>
       <c r="C38" s="19" t="s">
@@ -4382,16 +4412,16 @@
       <c r="Q38" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R38" s="180"/>
-      <c r="S38" s="154"/>
-      <c r="T38" s="154"/>
-      <c r="U38" s="154"/>
-      <c r="V38" s="154"/>
-      <c r="W38" s="155"/>
+      <c r="R38" s="202"/>
+      <c r="S38" s="169"/>
+      <c r="T38" s="169"/>
+      <c r="U38" s="169"/>
+      <c r="V38" s="169"/>
+      <c r="W38" s="170"/>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" s="59"/>
-      <c r="B39" s="163"/>
+      <c r="B39" s="166"/>
       <c r="C39" s="29" t="s">
         <v>12</v>
       </c>
@@ -4437,16 +4467,16 @@
       <c r="Q39" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R39" s="156"/>
-      <c r="S39" s="157"/>
-      <c r="T39" s="157"/>
-      <c r="U39" s="157"/>
-      <c r="V39" s="157"/>
-      <c r="W39" s="158"/>
+      <c r="R39" s="171"/>
+      <c r="S39" s="172"/>
+      <c r="T39" s="172"/>
+      <c r="U39" s="172"/>
+      <c r="V39" s="172"/>
+      <c r="W39" s="173"/>
     </row>
     <row r="40" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="59"/>
-      <c r="B40" s="166"/>
+      <c r="B40" s="167"/>
       <c r="C40" s="30" t="s">
         <v>14</v>
       </c>
@@ -4492,16 +4522,16 @@
       <c r="Q40" s="4">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R40" s="176"/>
-      <c r="S40" s="177"/>
-      <c r="T40" s="177"/>
-      <c r="U40" s="177"/>
-      <c r="V40" s="177"/>
-      <c r="W40" s="178"/>
+      <c r="R40" s="174"/>
+      <c r="S40" s="175"/>
+      <c r="T40" s="175"/>
+      <c r="U40" s="175"/>
+      <c r="V40" s="175"/>
+      <c r="W40" s="176"/>
     </row>
     <row r="41" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A41" s="59"/>
-      <c r="B41" s="162" t="s">
+      <c r="B41" s="165" t="s">
         <v>50</v>
       </c>
       <c r="C41" s="29" t="s">
@@ -4549,18 +4579,18 @@
       <c r="Q41" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R41" s="179" t="s">
+      <c r="R41" s="186" t="s">
         <v>71</v>
       </c>
-      <c r="S41" s="174"/>
-      <c r="T41" s="174"/>
-      <c r="U41" s="174"/>
-      <c r="V41" s="174"/>
-      <c r="W41" s="175"/>
+      <c r="S41" s="178"/>
+      <c r="T41" s="178"/>
+      <c r="U41" s="178"/>
+      <c r="V41" s="178"/>
+      <c r="W41" s="179"/>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A42" s="59"/>
-      <c r="B42" s="163"/>
+      <c r="B42" s="166"/>
       <c r="C42" s="29" t="s">
         <v>12</v>
       </c>
@@ -4606,16 +4636,16 @@
       <c r="Q42" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R42" s="167"/>
-      <c r="S42" s="168"/>
-      <c r="T42" s="168"/>
-      <c r="U42" s="168"/>
-      <c r="V42" s="168"/>
-      <c r="W42" s="169"/>
+      <c r="R42" s="180"/>
+      <c r="S42" s="181"/>
+      <c r="T42" s="181"/>
+      <c r="U42" s="181"/>
+      <c r="V42" s="181"/>
+      <c r="W42" s="182"/>
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A43" s="59"/>
-      <c r="B43" s="163"/>
+      <c r="B43" s="166"/>
       <c r="C43" s="29" t="s">
         <v>14</v>
       </c>
@@ -4661,16 +4691,16 @@
       <c r="Q43" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R43" s="167"/>
-      <c r="S43" s="168"/>
-      <c r="T43" s="168"/>
-      <c r="U43" s="168"/>
-      <c r="V43" s="168"/>
-      <c r="W43" s="169"/>
+      <c r="R43" s="180"/>
+      <c r="S43" s="181"/>
+      <c r="T43" s="181"/>
+      <c r="U43" s="181"/>
+      <c r="V43" s="181"/>
+      <c r="W43" s="182"/>
     </row>
     <row r="44" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="59"/>
-      <c r="B44" s="166"/>
+      <c r="B44" s="167"/>
       <c r="C44" s="30" t="s">
         <v>67</v>
       </c>
@@ -4716,16 +4746,16 @@
       <c r="Q44" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R44" s="170"/>
-      <c r="S44" s="171"/>
-      <c r="T44" s="171"/>
-      <c r="U44" s="171"/>
-      <c r="V44" s="171"/>
-      <c r="W44" s="172"/>
+      <c r="R44" s="183"/>
+      <c r="S44" s="184"/>
+      <c r="T44" s="184"/>
+      <c r="U44" s="184"/>
+      <c r="V44" s="184"/>
+      <c r="W44" s="185"/>
     </row>
     <row r="45" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A45" s="59"/>
-      <c r="B45" s="162" t="s">
+      <c r="B45" s="165" t="s">
         <v>55</v>
       </c>
       <c r="C45" s="29" t="s">
@@ -4773,18 +4803,18 @@
       <c r="Q45" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R45" s="153" t="s">
+      <c r="R45" s="168" t="s">
         <v>72</v>
       </c>
-      <c r="S45" s="154"/>
-      <c r="T45" s="154"/>
-      <c r="U45" s="154"/>
-      <c r="V45" s="154"/>
-      <c r="W45" s="155"/>
+      <c r="S45" s="169"/>
+      <c r="T45" s="169"/>
+      <c r="U45" s="169"/>
+      <c r="V45" s="169"/>
+      <c r="W45" s="170"/>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A46" s="59"/>
-      <c r="B46" s="163"/>
+      <c r="B46" s="166"/>
       <c r="C46" s="29" t="s">
         <v>12</v>
       </c>
@@ -4830,16 +4860,16 @@
       <c r="Q46" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R46" s="156"/>
-      <c r="S46" s="157"/>
-      <c r="T46" s="157"/>
-      <c r="U46" s="157"/>
-      <c r="V46" s="157"/>
-      <c r="W46" s="158"/>
+      <c r="R46" s="171"/>
+      <c r="S46" s="172"/>
+      <c r="T46" s="172"/>
+      <c r="U46" s="172"/>
+      <c r="V46" s="172"/>
+      <c r="W46" s="173"/>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A47" s="59"/>
-      <c r="B47" s="163"/>
+      <c r="B47" s="166"/>
       <c r="C47" s="29" t="s">
         <v>14</v>
       </c>
@@ -4885,16 +4915,16 @@
       <c r="Q47" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R47" s="156"/>
-      <c r="S47" s="157"/>
-      <c r="T47" s="157"/>
-      <c r="U47" s="157"/>
-      <c r="V47" s="157"/>
-      <c r="W47" s="158"/>
+      <c r="R47" s="171"/>
+      <c r="S47" s="172"/>
+      <c r="T47" s="172"/>
+      <c r="U47" s="172"/>
+      <c r="V47" s="172"/>
+      <c r="W47" s="173"/>
     </row>
     <row r="48" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="59"/>
-      <c r="B48" s="166"/>
+      <c r="B48" s="167"/>
       <c r="C48" s="30" t="s">
         <v>67</v>
       </c>
@@ -4940,16 +4970,16 @@
       <c r="Q48" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R48" s="176"/>
-      <c r="S48" s="177"/>
-      <c r="T48" s="177"/>
-      <c r="U48" s="177"/>
-      <c r="V48" s="177"/>
-      <c r="W48" s="178"/>
+      <c r="R48" s="174"/>
+      <c r="S48" s="175"/>
+      <c r="T48" s="175"/>
+      <c r="U48" s="175"/>
+      <c r="V48" s="175"/>
+      <c r="W48" s="176"/>
     </row>
     <row r="49" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A49" s="58"/>
-      <c r="B49" s="162" t="s">
+      <c r="B49" s="165" t="s">
         <v>58</v>
       </c>
       <c r="C49" s="29" t="s">
@@ -4997,18 +5027,18 @@
       <c r="Q49" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R49" s="173" t="s">
+      <c r="R49" s="177" t="s">
         <v>79</v>
       </c>
-      <c r="S49" s="174"/>
-      <c r="T49" s="174"/>
-      <c r="U49" s="174"/>
-      <c r="V49" s="174"/>
-      <c r="W49" s="175"/>
+      <c r="S49" s="178"/>
+      <c r="T49" s="178"/>
+      <c r="U49" s="178"/>
+      <c r="V49" s="178"/>
+      <c r="W49" s="179"/>
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A50" s="58"/>
-      <c r="B50" s="163"/>
+      <c r="B50" s="166"/>
       <c r="C50" s="29" t="s">
         <v>12</v>
       </c>
@@ -5054,16 +5084,16 @@
       <c r="Q50" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R50" s="167"/>
-      <c r="S50" s="168"/>
-      <c r="T50" s="168"/>
-      <c r="U50" s="168"/>
-      <c r="V50" s="168"/>
-      <c r="W50" s="169"/>
+      <c r="R50" s="180"/>
+      <c r="S50" s="181"/>
+      <c r="T50" s="181"/>
+      <c r="U50" s="181"/>
+      <c r="V50" s="181"/>
+      <c r="W50" s="182"/>
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A51" s="58"/>
-      <c r="B51" s="163"/>
+      <c r="B51" s="166"/>
       <c r="C51" s="29" t="s">
         <v>14</v>
       </c>
@@ -5109,16 +5139,16 @@
       <c r="Q51" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R51" s="167"/>
-      <c r="S51" s="168"/>
-      <c r="T51" s="168"/>
-      <c r="U51" s="168"/>
-      <c r="V51" s="168"/>
-      <c r="W51" s="169"/>
+      <c r="R51" s="180"/>
+      <c r="S51" s="181"/>
+      <c r="T51" s="181"/>
+      <c r="U51" s="181"/>
+      <c r="V51" s="181"/>
+      <c r="W51" s="182"/>
     </row>
     <row r="52" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="58"/>
-      <c r="B52" s="166"/>
+      <c r="B52" s="167"/>
       <c r="C52" s="30" t="s">
         <v>67</v>
       </c>
@@ -5164,16 +5194,16 @@
       <c r="Q52" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R52" s="170"/>
-      <c r="S52" s="171"/>
-      <c r="T52" s="171"/>
-      <c r="U52" s="171"/>
-      <c r="V52" s="171"/>
-      <c r="W52" s="172"/>
+      <c r="R52" s="183"/>
+      <c r="S52" s="184"/>
+      <c r="T52" s="184"/>
+      <c r="U52" s="184"/>
+      <c r="V52" s="184"/>
+      <c r="W52" s="185"/>
     </row>
     <row r="53" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A53" s="59"/>
-      <c r="B53" s="162" t="s">
+      <c r="B53" s="165" t="s">
         <v>77</v>
       </c>
       <c r="C53" s="19" t="s">
@@ -5221,18 +5251,18 @@
       <c r="Q53" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R53" s="173" t="s">
+      <c r="R53" s="177" t="s">
         <v>80</v>
       </c>
-      <c r="S53" s="174"/>
-      <c r="T53" s="174"/>
-      <c r="U53" s="174"/>
-      <c r="V53" s="174"/>
-      <c r="W53" s="175"/>
+      <c r="S53" s="178"/>
+      <c r="T53" s="178"/>
+      <c r="U53" s="178"/>
+      <c r="V53" s="178"/>
+      <c r="W53" s="179"/>
     </row>
     <row r="54" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A54" s="59"/>
-      <c r="B54" s="163"/>
+      <c r="B54" s="166"/>
       <c r="C54" s="29" t="s">
         <v>12</v>
       </c>
@@ -5278,16 +5308,16 @@
       <c r="Q54" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R54" s="167"/>
-      <c r="S54" s="168"/>
-      <c r="T54" s="168"/>
-      <c r="U54" s="168"/>
-      <c r="V54" s="168"/>
-      <c r="W54" s="169"/>
+      <c r="R54" s="180"/>
+      <c r="S54" s="181"/>
+      <c r="T54" s="181"/>
+      <c r="U54" s="181"/>
+      <c r="V54" s="181"/>
+      <c r="W54" s="182"/>
     </row>
     <row r="55" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A55" s="59"/>
-      <c r="B55" s="163"/>
+      <c r="B55" s="166"/>
       <c r="C55" s="29" t="s">
         <v>14</v>
       </c>
@@ -5333,16 +5363,16 @@
       <c r="Q55" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R55" s="167"/>
-      <c r="S55" s="168"/>
-      <c r="T55" s="168"/>
-      <c r="U55" s="168"/>
-      <c r="V55" s="168"/>
-      <c r="W55" s="169"/>
+      <c r="R55" s="180"/>
+      <c r="S55" s="181"/>
+      <c r="T55" s="181"/>
+      <c r="U55" s="181"/>
+      <c r="V55" s="181"/>
+      <c r="W55" s="182"/>
     </row>
     <row r="56" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A56" s="59"/>
-      <c r="B56" s="166"/>
+      <c r="B56" s="167"/>
       <c r="C56" s="30" t="s">
         <v>67</v>
       </c>
@@ -5388,16 +5418,16 @@
       <c r="Q56" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R56" s="170"/>
-      <c r="S56" s="171"/>
-      <c r="T56" s="171"/>
-      <c r="U56" s="171"/>
-      <c r="V56" s="171"/>
-      <c r="W56" s="172"/>
+      <c r="R56" s="183"/>
+      <c r="S56" s="184"/>
+      <c r="T56" s="184"/>
+      <c r="U56" s="184"/>
+      <c r="V56" s="184"/>
+      <c r="W56" s="185"/>
     </row>
     <row r="57" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A57" s="58"/>
-      <c r="B57" s="162" t="s">
+      <c r="B57" s="165" t="s">
         <v>81</v>
       </c>
       <c r="C57" s="19" t="s">
@@ -5445,18 +5475,18 @@
       <c r="Q57" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R57" s="173" t="s">
+      <c r="R57" s="177" t="s">
         <v>87</v>
       </c>
-      <c r="S57" s="174"/>
-      <c r="T57" s="174"/>
-      <c r="U57" s="174"/>
-      <c r="V57" s="174"/>
-      <c r="W57" s="175"/>
+      <c r="S57" s="178"/>
+      <c r="T57" s="178"/>
+      <c r="U57" s="178"/>
+      <c r="V57" s="178"/>
+      <c r="W57" s="179"/>
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A58" s="58"/>
-      <c r="B58" s="163"/>
+      <c r="B58" s="166"/>
       <c r="C58" s="29" t="s">
         <v>12</v>
       </c>
@@ -5502,16 +5532,16 @@
       <c r="Q58" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R58" s="167"/>
-      <c r="S58" s="168"/>
-      <c r="T58" s="168"/>
-      <c r="U58" s="168"/>
-      <c r="V58" s="168"/>
-      <c r="W58" s="169"/>
+      <c r="R58" s="180"/>
+      <c r="S58" s="181"/>
+      <c r="T58" s="181"/>
+      <c r="U58" s="181"/>
+      <c r="V58" s="181"/>
+      <c r="W58" s="182"/>
     </row>
     <row r="59" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A59" s="58"/>
-      <c r="B59" s="163"/>
+      <c r="B59" s="166"/>
       <c r="C59" s="29" t="s">
         <v>14</v>
       </c>
@@ -5557,16 +5587,16 @@
       <c r="Q59" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R59" s="167"/>
-      <c r="S59" s="168"/>
-      <c r="T59" s="168"/>
-      <c r="U59" s="168"/>
-      <c r="V59" s="168"/>
-      <c r="W59" s="169"/>
+      <c r="R59" s="180"/>
+      <c r="S59" s="181"/>
+      <c r="T59" s="181"/>
+      <c r="U59" s="181"/>
+      <c r="V59" s="181"/>
+      <c r="W59" s="182"/>
     </row>
     <row r="60" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="58"/>
-      <c r="B60" s="166"/>
+      <c r="B60" s="167"/>
       <c r="C60" s="30" t="s">
         <v>67</v>
       </c>
@@ -5612,16 +5642,16 @@
       <c r="Q60" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R60" s="170"/>
-      <c r="S60" s="171"/>
-      <c r="T60" s="171"/>
-      <c r="U60" s="171"/>
-      <c r="V60" s="171"/>
-      <c r="W60" s="172"/>
+      <c r="R60" s="183"/>
+      <c r="S60" s="184"/>
+      <c r="T60" s="184"/>
+      <c r="U60" s="184"/>
+      <c r="V60" s="184"/>
+      <c r="W60" s="185"/>
     </row>
     <row r="61" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A61" s="7"/>
-      <c r="B61" s="162" t="s">
+      <c r="B61" s="165" t="s">
         <v>84</v>
       </c>
       <c r="C61" s="28" t="s">
@@ -5669,18 +5699,18 @@
       <c r="Q61" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R61" s="153" t="s">
+      <c r="R61" s="168" t="s">
         <v>85</v>
       </c>
-      <c r="S61" s="154"/>
-      <c r="T61" s="154"/>
-      <c r="U61" s="154"/>
-      <c r="V61" s="154"/>
-      <c r="W61" s="155"/>
+      <c r="S61" s="169"/>
+      <c r="T61" s="169"/>
+      <c r="U61" s="169"/>
+      <c r="V61" s="169"/>
+      <c r="W61" s="170"/>
     </row>
     <row r="62" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A62" s="7"/>
-      <c r="B62" s="163"/>
+      <c r="B62" s="166"/>
       <c r="C62" s="25" t="s">
         <v>12</v>
       </c>
@@ -5726,16 +5756,16 @@
       <c r="Q62" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R62" s="156"/>
-      <c r="S62" s="157"/>
-      <c r="T62" s="157"/>
-      <c r="U62" s="157"/>
-      <c r="V62" s="157"/>
-      <c r="W62" s="158"/>
+      <c r="R62" s="171"/>
+      <c r="S62" s="172"/>
+      <c r="T62" s="172"/>
+      <c r="U62" s="172"/>
+      <c r="V62" s="172"/>
+      <c r="W62" s="173"/>
     </row>
     <row r="63" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="163"/>
+      <c r="B63" s="166"/>
       <c r="C63" s="25" t="s">
         <v>14</v>
       </c>
@@ -5781,16 +5811,16 @@
       <c r="Q63" s="64">
         <v>1E-3</v>
       </c>
-      <c r="R63" s="156"/>
-      <c r="S63" s="157"/>
-      <c r="T63" s="157"/>
-      <c r="U63" s="157"/>
-      <c r="V63" s="157"/>
-      <c r="W63" s="158"/>
+      <c r="R63" s="171"/>
+      <c r="S63" s="172"/>
+      <c r="T63" s="172"/>
+      <c r="U63" s="172"/>
+      <c r="V63" s="172"/>
+      <c r="W63" s="173"/>
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="163"/>
+      <c r="B64" s="166"/>
       <c r="C64" s="25" t="s">
         <v>67</v>
       </c>
@@ -5836,16 +5866,16 @@
       <c r="Q64" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R64" s="156"/>
-      <c r="S64" s="157"/>
-      <c r="T64" s="157"/>
-      <c r="U64" s="157"/>
-      <c r="V64" s="157"/>
-      <c r="W64" s="158"/>
+      <c r="R64" s="171"/>
+      <c r="S64" s="172"/>
+      <c r="T64" s="172"/>
+      <c r="U64" s="172"/>
+      <c r="V64" s="172"/>
+      <c r="W64" s="173"/>
     </row>
     <row r="65" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="7"/>
-      <c r="B65" s="166"/>
+      <c r="B65" s="167"/>
       <c r="C65" s="67" t="s">
         <v>83</v>
       </c>
@@ -5891,15 +5921,15 @@
       <c r="Q65" s="69">
         <v>1E-3</v>
       </c>
-      <c r="R65" s="176"/>
-      <c r="S65" s="177"/>
-      <c r="T65" s="177"/>
-      <c r="U65" s="177"/>
-      <c r="V65" s="177"/>
-      <c r="W65" s="178"/>
+      <c r="R65" s="174"/>
+      <c r="S65" s="175"/>
+      <c r="T65" s="175"/>
+      <c r="U65" s="175"/>
+      <c r="V65" s="175"/>
+      <c r="W65" s="176"/>
     </row>
     <row r="66" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B66" s="162" t="s">
+      <c r="B66" s="165" t="s">
         <v>86</v>
       </c>
       <c r="C66" s="19" t="s">
@@ -5947,17 +5977,17 @@
       <c r="Q66" s="9">
         <v>1E-3</v>
       </c>
-      <c r="R66" s="153" t="s">
+      <c r="R66" s="168" t="s">
         <v>88</v>
       </c>
-      <c r="S66" s="154"/>
-      <c r="T66" s="154"/>
-      <c r="U66" s="154"/>
-      <c r="V66" s="154"/>
-      <c r="W66" s="155"/>
+      <c r="S66" s="169"/>
+      <c r="T66" s="169"/>
+      <c r="U66" s="169"/>
+      <c r="V66" s="169"/>
+      <c r="W66" s="170"/>
     </row>
     <row r="67" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B67" s="163"/>
+      <c r="B67" s="166"/>
       <c r="C67" s="29" t="s">
         <v>12</v>
       </c>
@@ -6003,15 +6033,15 @@
       <c r="Q67" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R67" s="156"/>
-      <c r="S67" s="157"/>
-      <c r="T67" s="157"/>
-      <c r="U67" s="157"/>
-      <c r="V67" s="157"/>
-      <c r="W67" s="158"/>
+      <c r="R67" s="171"/>
+      <c r="S67" s="172"/>
+      <c r="T67" s="172"/>
+      <c r="U67" s="172"/>
+      <c r="V67" s="172"/>
+      <c r="W67" s="173"/>
     </row>
     <row r="68" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B68" s="163"/>
+      <c r="B68" s="166"/>
       <c r="C68" s="29" t="s">
         <v>14</v>
       </c>
@@ -6057,15 +6087,15 @@
       <c r="Q68" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R68" s="156"/>
-      <c r="S68" s="157"/>
-      <c r="T68" s="157"/>
-      <c r="U68" s="157"/>
-      <c r="V68" s="157"/>
-      <c r="W68" s="158"/>
+      <c r="R68" s="171"/>
+      <c r="S68" s="172"/>
+      <c r="T68" s="172"/>
+      <c r="U68" s="172"/>
+      <c r="V68" s="172"/>
+      <c r="W68" s="173"/>
     </row>
     <row r="69" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="164"/>
+      <c r="B69" s="206"/>
       <c r="C69" s="29" t="s">
         <v>67</v>
       </c>
@@ -6111,15 +6141,15 @@
       <c r="Q69" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R69" s="159"/>
-      <c r="S69" s="160"/>
-      <c r="T69" s="160"/>
-      <c r="U69" s="160"/>
-      <c r="V69" s="160"/>
-      <c r="W69" s="161"/>
+      <c r="R69" s="203"/>
+      <c r="S69" s="204"/>
+      <c r="T69" s="204"/>
+      <c r="U69" s="204"/>
+      <c r="V69" s="204"/>
+      <c r="W69" s="205"/>
     </row>
     <row r="70" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B70" s="165" t="s">
+      <c r="B70" s="207" t="s">
         <v>89</v>
       </c>
       <c r="C70" s="72" t="s">
@@ -6167,17 +6197,17 @@
       <c r="Q70" s="16">
         <v>1E-3</v>
       </c>
-      <c r="R70" s="167" t="s">
+      <c r="R70" s="180" t="s">
         <v>90</v>
       </c>
-      <c r="S70" s="168"/>
-      <c r="T70" s="168"/>
-      <c r="U70" s="168"/>
-      <c r="V70" s="168"/>
-      <c r="W70" s="169"/>
+      <c r="S70" s="181"/>
+      <c r="T70" s="181"/>
+      <c r="U70" s="181"/>
+      <c r="V70" s="181"/>
+      <c r="W70" s="182"/>
     </row>
     <row r="71" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B71" s="163"/>
+      <c r="B71" s="166"/>
       <c r="C71" s="29" t="s">
         <v>12</v>
       </c>
@@ -6223,15 +6253,15 @@
       <c r="Q71" s="7">
         <v>1E-3</v>
       </c>
-      <c r="R71" s="167"/>
-      <c r="S71" s="168"/>
-      <c r="T71" s="168"/>
-      <c r="U71" s="168"/>
-      <c r="V71" s="168"/>
-      <c r="W71" s="169"/>
+      <c r="R71" s="180"/>
+      <c r="S71" s="181"/>
+      <c r="T71" s="181"/>
+      <c r="U71" s="181"/>
+      <c r="V71" s="181"/>
+      <c r="W71" s="182"/>
     </row>
     <row r="72" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="B72" s="163"/>
+      <c r="B72" s="166"/>
       <c r="C72" s="29" t="s">
         <v>14</v>
       </c>
@@ -6277,15 +6307,15 @@
       <c r="Q72" s="7">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="R72" s="167"/>
-      <c r="S72" s="168"/>
-      <c r="T72" s="168"/>
-      <c r="U72" s="168"/>
-      <c r="V72" s="168"/>
-      <c r="W72" s="169"/>
+      <c r="R72" s="180"/>
+      <c r="S72" s="181"/>
+      <c r="T72" s="181"/>
+      <c r="U72" s="181"/>
+      <c r="V72" s="181"/>
+      <c r="W72" s="182"/>
     </row>
     <row r="73" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="166"/>
+      <c r="B73" s="167"/>
       <c r="C73" s="30" t="s">
         <v>67</v>
       </c>
@@ -6331,16 +6361,43 @@
       <c r="Q73" s="4">
         <v>1E-3</v>
       </c>
-      <c r="R73" s="170"/>
-      <c r="S73" s="171"/>
-      <c r="T73" s="171"/>
-      <c r="U73" s="171"/>
-      <c r="V73" s="171"/>
-      <c r="W73" s="172"/>
+      <c r="R73" s="183"/>
+      <c r="S73" s="184"/>
+      <c r="T73" s="184"/>
+      <c r="U73" s="184"/>
+      <c r="V73" s="184"/>
+      <c r="W73" s="185"/>
     </row>
     <row r="74" spans="1:23" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="43">
+    <mergeCell ref="R66:W69"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="R70:W73"/>
+    <mergeCell ref="B53:B56"/>
+    <mergeCell ref="R53:W56"/>
+    <mergeCell ref="R45:W48"/>
+    <mergeCell ref="B45:B48"/>
+    <mergeCell ref="R49:W52"/>
+    <mergeCell ref="B49:B52"/>
+    <mergeCell ref="R23:W25"/>
+    <mergeCell ref="B26:B28"/>
+    <mergeCell ref="R26:W28"/>
+    <mergeCell ref="B23:B25"/>
+    <mergeCell ref="B38:B40"/>
+    <mergeCell ref="R38:W40"/>
+    <mergeCell ref="B35:B37"/>
+    <mergeCell ref="R35:W37"/>
+    <mergeCell ref="B41:B44"/>
+    <mergeCell ref="R41:W44"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="I3:Q3"/>
+    <mergeCell ref="B5:B7"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="R3:W4"/>
+    <mergeCell ref="R5:W7"/>
+    <mergeCell ref="R8:W10"/>
     <mergeCell ref="B11:B13"/>
     <mergeCell ref="B61:B65"/>
     <mergeCell ref="R61:W65"/>
@@ -6357,33 +6414,6 @@
     <mergeCell ref="R29:W31"/>
     <mergeCell ref="B32:B34"/>
     <mergeCell ref="R32:W34"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="I3:Q3"/>
-    <mergeCell ref="B5:B7"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="R3:W4"/>
-    <mergeCell ref="R5:W7"/>
-    <mergeCell ref="R8:W10"/>
-    <mergeCell ref="R45:W48"/>
-    <mergeCell ref="B45:B48"/>
-    <mergeCell ref="R49:W52"/>
-    <mergeCell ref="B49:B52"/>
-    <mergeCell ref="R23:W25"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="R26:W28"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="B38:B40"/>
-    <mergeCell ref="R38:W40"/>
-    <mergeCell ref="B35:B37"/>
-    <mergeCell ref="R35:W37"/>
-    <mergeCell ref="B41:B44"/>
-    <mergeCell ref="R41:W44"/>
-    <mergeCell ref="R66:W69"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="B70:B73"/>
-    <mergeCell ref="R70:W73"/>
-    <mergeCell ref="B53:B56"/>
-    <mergeCell ref="R53:W56"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
@@ -6397,17 +6427,17 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="204" t="s">
+      <c r="B2" s="214" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="204"/>
-      <c r="D2" s="204"/>
-      <c r="E2" s="204"/>
-      <c r="F2" s="204"/>
-      <c r="G2" s="204"/>
-      <c r="H2" s="204"/>
-      <c r="I2" s="204"/>
-      <c r="J2" s="204"/>
+      <c r="C2" s="214"/>
+      <c r="D2" s="214"/>
+      <c r="E2" s="214"/>
+      <c r="F2" s="214"/>
+      <c r="G2" s="214"/>
+      <c r="H2" s="214"/>
+      <c r="I2" s="214"/>
+      <c r="J2" s="214"/>
     </row>
     <row r="4" spans="2:10" x14ac:dyDescent="0.25">
       <c r="C4" s="116"/>
@@ -6431,7 +6461,7 @@
       </c>
     </row>
     <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="201" t="s">
+      <c r="B5" s="211" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="133" t="s">
@@ -6457,7 +6487,7 @@
       </c>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="202"/>
+      <c r="B6" s="212"/>
       <c r="C6" s="136" t="s">
         <v>97</v>
       </c>
@@ -6481,7 +6511,7 @@
       </c>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="203" t="s">
+      <c r="B7" s="213" t="s">
         <v>14</v>
       </c>
       <c r="C7" s="117" t="s">
@@ -6507,7 +6537,7 @@
       </c>
     </row>
     <row r="8" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B8" s="202"/>
+      <c r="B8" s="212"/>
       <c r="C8" s="136" t="s">
         <v>97</v>
       </c>
@@ -6562,17 +6592,17 @@
       </c>
     </row>
     <row r="14" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B14" s="204" t="s">
+      <c r="B14" s="214" t="s">
         <v>101</v>
       </c>
-      <c r="C14" s="204"/>
-      <c r="D14" s="204"/>
-      <c r="E14" s="204"/>
-      <c r="F14" s="204"/>
-      <c r="G14" s="204"/>
-      <c r="H14" s="204"/>
-      <c r="I14" s="204"/>
-      <c r="J14" s="204"/>
+      <c r="C14" s="214"/>
+      <c r="D14" s="214"/>
+      <c r="E14" s="214"/>
+      <c r="F14" s="214"/>
+      <c r="G14" s="214"/>
+      <c r="H14" s="214"/>
+      <c r="I14" s="214"/>
+      <c r="J14" s="214"/>
     </row>
     <row r="15" spans="2:10" x14ac:dyDescent="0.25">
       <c r="D15" s="124"/>
@@ -6606,7 +6636,7 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="129"/>
-      <c r="B17" s="205" t="s">
+      <c r="B17" s="215" t="s">
         <v>12</v>
       </c>
       <c r="C17" s="123" t="s">
@@ -6633,7 +6663,7 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="129"/>
-      <c r="B18" s="206"/>
+      <c r="B18" s="216"/>
       <c r="C18" s="121" t="s">
         <v>97</v>
       </c>
@@ -6658,7 +6688,7 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="129"/>
-      <c r="B19" s="205" t="s">
+      <c r="B19" s="215" t="s">
         <v>14</v>
       </c>
       <c r="C19" s="119" t="s">
@@ -6685,7 +6715,7 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="129"/>
-      <c r="B20" s="206"/>
+      <c r="B20" s="216"/>
       <c r="C20" s="121" t="s">
         <v>97</v>
       </c>
@@ -6739,17 +6769,17 @@
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B26" s="204" t="s">
+      <c r="B26" s="214" t="s">
         <v>102</v>
       </c>
-      <c r="C26" s="204"/>
-      <c r="D26" s="204"/>
-      <c r="E26" s="204"/>
-      <c r="F26" s="204"/>
-      <c r="G26" s="204"/>
-      <c r="H26" s="204"/>
-      <c r="I26" s="204"/>
-      <c r="J26" s="204"/>
+      <c r="C26" s="214"/>
+      <c r="D26" s="214"/>
+      <c r="E26" s="214"/>
+      <c r="F26" s="214"/>
+      <c r="G26" s="214"/>
+      <c r="H26" s="214"/>
+      <c r="I26" s="214"/>
+      <c r="J26" s="214"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="C28" s="116"/>
@@ -6773,7 +6803,7 @@
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B29" s="198" t="s">
+      <c r="B29" s="208" t="s">
         <v>12</v>
       </c>
       <c r="C29" s="137" t="s">
@@ -6799,7 +6829,7 @@
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B30" s="199"/>
+      <c r="B30" s="209"/>
       <c r="C30" s="138" t="s">
         <v>97</v>
       </c>
@@ -6823,7 +6853,7 @@
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B31" s="200" t="s">
+      <c r="B31" s="210" t="s">
         <v>14</v>
       </c>
       <c r="C31" s="120" t="s">
@@ -6849,7 +6879,7 @@
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B32" s="199"/>
+      <c r="B32" s="209"/>
       <c r="C32" s="138" t="s">
         <v>97</v>
       </c>
@@ -6928,13 +6958,13 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B3" s="207" t="s">
+      <c r="B3" s="217" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="207"/>
-      <c r="D3" s="207"/>
-      <c r="E3" s="207"/>
-      <c r="F3" s="207"/>
+      <c r="C3" s="217"/>
+      <c r="D3" s="217"/>
+      <c r="E3" s="217"/>
+      <c r="F3" s="217"/>
     </row>
     <row r="5" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="90"/>
@@ -6968,30 +6998,30 @@
       </c>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B25" s="207" t="s">
+      <c r="B25" s="217" t="s">
         <v>104</v>
       </c>
-      <c r="C25" s="207"/>
-      <c r="D25" s="207"/>
-      <c r="E25" s="207"/>
-      <c r="F25" s="207"/>
-      <c r="G25" s="207"/>
-      <c r="H25" s="207"/>
-      <c r="I25" s="207"/>
-      <c r="J25" s="207"/>
+      <c r="C25" s="217"/>
+      <c r="D25" s="217"/>
+      <c r="E25" s="217"/>
+      <c r="F25" s="217"/>
+      <c r="G25" s="217"/>
+      <c r="H25" s="217"/>
+      <c r="I25" s="217"/>
+      <c r="J25" s="217"/>
     </row>
     <row r="27" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B27" s="208" t="s">
+      <c r="B27" s="218" t="s">
         <v>110</v>
       </c>
-      <c r="C27" s="209"/>
-      <c r="D27" s="209"/>
-      <c r="E27" s="209"/>
-      <c r="F27" s="209"/>
-      <c r="G27" s="209"/>
-      <c r="H27" s="209"/>
-      <c r="I27" s="209"/>
-      <c r="J27" s="210"/>
+      <c r="C27" s="219"/>
+      <c r="D27" s="219"/>
+      <c r="E27" s="219"/>
+      <c r="F27" s="219"/>
+      <c r="G27" s="219"/>
+      <c r="H27" s="219"/>
+      <c r="I27" s="219"/>
+      <c r="J27" s="220"/>
     </row>
     <row r="28" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B28" s="77" t="s">
@@ -7168,17 +7198,17 @@
       </c>
     </row>
     <row r="35" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B35" s="211" t="s">
+      <c r="B35" s="221" t="s">
         <v>116</v>
       </c>
-      <c r="C35" s="212"/>
-      <c r="D35" s="212"/>
-      <c r="E35" s="212"/>
-      <c r="F35" s="212"/>
-      <c r="G35" s="212"/>
-      <c r="H35" s="212"/>
-      <c r="I35" s="212"/>
-      <c r="J35" s="213"/>
+      <c r="C35" s="222"/>
+      <c r="D35" s="222"/>
+      <c r="E35" s="222"/>
+      <c r="F35" s="222"/>
+      <c r="G35" s="222"/>
+      <c r="H35" s="222"/>
+      <c r="I35" s="222"/>
+      <c r="J35" s="223"/>
     </row>
     <row r="36" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B36" s="84" t="s">
@@ -7369,45 +7399,47 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49131BC2-9475-4600-9F3F-41F4402E55A0}">
-  <dimension ref="B8:E13"/>
+  <dimension ref="B8:L18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.42578125" customWidth="1"/>
     <col min="3" max="3" width="17" customWidth="1"/>
     <col min="4" max="4" width="19.5703125" customWidth="1"/>
     <col min="5" max="5" width="17.85546875" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" customWidth="1"/>
+    <col min="12" max="12" width="9.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="2:5" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="214" t="s">
+    <row r="8" spans="2:12" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="153" t="s">
         <v>119</v>
       </c>
-      <c r="C8" s="214" t="s">
+      <c r="C8" s="153" t="s">
         <v>120</v>
       </c>
-      <c r="D8" s="214" t="s">
+      <c r="D8" s="153" t="s">
         <v>121</v>
       </c>
-      <c r="E8" s="214" t="s">
+      <c r="E8" s="153" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="215" t="s">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B9" s="154" t="s">
         <v>117</v>
       </c>
-      <c r="C9" s="216">
+      <c r="C9" s="155">
         <v>1680</v>
       </c>
-      <c r="D9" s="216">
+      <c r="D9" s="155">
         <v>1680</v>
       </c>
-      <c r="E9" s="216">
+      <c r="E9" s="155">
         <v>738</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B10" s="215" t="s">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B10" s="154" t="s">
         <v>91</v>
       </c>
       <c r="C10" s="31" t="s">
@@ -7420,22 +7452,22 @@
         <v>127</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="215" t="s">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B11" s="154" t="s">
         <v>93</v>
       </c>
-      <c r="C11" s="216" t="s">
+      <c r="C11" s="155" t="s">
         <v>124</v>
       </c>
-      <c r="D11" s="216" t="s">
+      <c r="D11" s="155" t="s">
         <v>126</v>
       </c>
-      <c r="E11" s="216" t="s">
+      <c r="E11" s="155" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B12" s="215" t="s">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B12" s="154" t="s">
         <v>2</v>
       </c>
       <c r="C12" s="31">
@@ -7448,21 +7480,107 @@
         <v>0.85109999999999997</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B13" s="215" t="s">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B13" s="154" t="s">
         <v>118</v>
       </c>
-      <c r="C13" s="216">
+      <c r="C13" s="155">
         <v>-21.3919</v>
       </c>
-      <c r="D13" s="216">
+      <c r="D13" s="155">
         <v>0.91690000000000005</v>
       </c>
-      <c r="E13" s="216">
+      <c r="E13" s="155">
         <v>0.84840000000000004</v>
       </c>
     </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="G14" s="161" t="s">
+        <v>129</v>
+      </c>
+      <c r="H14" s="161"/>
+      <c r="I14" s="161"/>
+      <c r="J14" s="157" t="s">
+        <v>22</v>
+      </c>
+      <c r="K14" s="157" t="s">
+        <v>23</v>
+      </c>
+      <c r="L14" s="157" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="G15" s="162" t="s">
+        <v>130</v>
+      </c>
+      <c r="H15" s="162"/>
+      <c r="I15" s="162"/>
+      <c r="J15" s="156">
+        <v>71.099999999999994</v>
+      </c>
+      <c r="K15" s="156">
+        <v>134</v>
+      </c>
+      <c r="L15" s="158">
+        <v>0.89500000000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="G16" s="162" t="s">
+        <v>133</v>
+      </c>
+      <c r="H16" s="162"/>
+      <c r="I16" s="162"/>
+      <c r="J16">
+        <v>46.22</v>
+      </c>
+      <c r="K16">
+        <v>71.78</v>
+      </c>
+      <c r="L16">
+        <v>0.93140000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="G17" s="162" t="s">
+        <v>131</v>
+      </c>
+      <c r="H17" s="162"/>
+      <c r="I17" s="162"/>
+      <c r="J17" s="156">
+        <v>46.23</v>
+      </c>
+      <c r="K17" s="156">
+        <v>94.53</v>
+      </c>
+      <c r="L17" s="158">
+        <v>0.86029999999999995</v>
+      </c>
+    </row>
+    <row r="18" spans="7:12" x14ac:dyDescent="0.25">
+      <c r="G18" s="159" t="s">
+        <v>132</v>
+      </c>
+      <c r="H18" s="159"/>
+      <c r="I18" s="159"/>
+      <c r="J18">
+        <v>84.05</v>
+      </c>
+      <c r="K18">
+        <v>129.25</v>
+      </c>
+      <c r="L18" s="160">
+        <v>0.6694</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="G15:I15"/>
+    <mergeCell ref="G17:I17"/>
+    <mergeCell ref="G16:I16"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>